<commit_message>
fix(auth): address registration review findings
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R1f36bd92c5a04753"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R0464abf6bbab4e51"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -141,9 +141,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -304,204 +304,84 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="11" t="str">
-        <x:v>2026-06-29</x:v>
-      </x:c>
-      <x:c r="B2" s="11" t="str">
-        <x:v>17:10</x:v>
-      </x:c>
-      <x:c r="C2" s="11" t="str">
-        <x:v>DOC-001</x:v>
-      </x:c>
-      <x:c r="D2" s="11" t="str">
-        <x:v>Documentation</x:v>
-      </x:c>
-      <x:c r="E2" s="11" t="str">
-        <x:v>CHANGE_LOG.md</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="str">
-        <x:v>新增</x:v>
-      </x:c>
-      <x:c r="G2" s="11" t="str">
-        <x:v>建立文字版專案異動紀錄</x:v>
-      </x:c>
-      <x:c r="H2" s="11" t="str">
-        <x:v>ChatGPT</x:v>
-      </x:c>
-      <x:c r="I2" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="J2" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K2" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L2" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="M2" s="11" t="str"/>
+      <x:c r="A2" s="11"/>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+      <x:c r="G2" s="11"/>
+      <x:c r="H2" s="11"/>
+      <x:c r="I2" s="11"/>
+      <x:c r="J2" s="11"/>
+      <x:c r="K2" s="11"/>
+      <x:c r="L2" s="11"/>
+      <x:c r="M2" s="11"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="11" t="str">
-        <x:v>2026-06-29</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="str">
-        <x:v>17:10</x:v>
-      </x:c>
-      <x:c r="C3" s="11" t="str">
-        <x:v>DOC-001</x:v>
-      </x:c>
-      <x:c r="D3" s="11" t="str">
-        <x:v>Documentation</x:v>
-      </x:c>
-      <x:c r="E3" s="11" t="str">
-        <x:v>CHANGE_HISTORY.csv</x:v>
-      </x:c>
-      <x:c r="F3" s="11" t="str">
-        <x:v>新增</x:v>
-      </x:c>
-      <x:c r="G3" s="11" t="str">
-        <x:v>建立 CSV 版專案異動歷程</x:v>
-      </x:c>
-      <x:c r="H3" s="11" t="str">
-        <x:v>ChatGPT</x:v>
-      </x:c>
-      <x:c r="I3" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="J3" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K3" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L3" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="M3" s="11" t="str"/>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="11"/>
+      <x:c r="C3" s="11"/>
+      <x:c r="D3" s="11"/>
+      <x:c r="E3" s="11"/>
+      <x:c r="F3" s="11"/>
+      <x:c r="G3" s="11"/>
+      <x:c r="H3" s="11"/>
+      <x:c r="I3" s="11"/>
+      <x:c r="J3" s="11"/>
+      <x:c r="K3" s="11"/>
+      <x:c r="L3" s="11"/>
+      <x:c r="M3" s="11"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="11" t="str">
-        <x:v>2026-06-29</x:v>
-      </x:c>
-      <x:c r="B4" s="11" t="str">
-        <x:v>17:10</x:v>
-      </x:c>
-      <x:c r="C4" s="11" t="str">
-        <x:v>DOC-001</x:v>
-      </x:c>
-      <x:c r="D4" s="11" t="str">
-        <x:v>Documentation</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="str">
-        <x:v>CHANGE_HISTORY.xlsx</x:v>
-      </x:c>
-      <x:c r="F4" s="11" t="str">
-        <x:v>新增</x:v>
-      </x:c>
-      <x:c r="G4" s="11" t="str">
-        <x:v>建立 Excel 版專案異動歷程</x:v>
-      </x:c>
-      <x:c r="H4" s="11" t="str">
-        <x:v>ChatGPT</x:v>
-      </x:c>
-      <x:c r="I4" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="J4" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K4" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L4" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="M4" s="11" t="str"/>
+      <x:c r="A4" s="11"/>
+      <x:c r="B4" s="11"/>
+      <x:c r="C4" s="11"/>
+      <x:c r="D4" s="11"/>
+      <x:c r="E4" s="11"/>
+      <x:c r="F4" s="11"/>
+      <x:c r="G4" s="11"/>
+      <x:c r="H4" s="11"/>
+      <x:c r="I4" s="11"/>
+      <x:c r="J4" s="11"/>
+      <x:c r="K4" s="11"/>
+      <x:c r="L4" s="11"/>
+      <x:c r="M4" s="11"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="11" t="str">
-        <x:v>2026-06-29</x:v>
-      </x:c>
-      <x:c r="B5" s="11" t="str">
-        <x:v>17:10</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="str">
-        <x:v>DOC-001</x:v>
-      </x:c>
-      <x:c r="D5" s="11" t="str">
-        <x:v>Documentation</x:v>
-      </x:c>
-      <x:c r="E5" s="11" t="str">
-        <x:v>README.md</x:v>
-      </x:c>
-      <x:c r="F5" s="11" t="str">
-        <x:v>修改</x:v>
-      </x:c>
-      <x:c r="G5" s="11" t="str">
-        <x:v>更新 AI Coding Agent 使用指令與文件閱讀順序</x:v>
-      </x:c>
-      <x:c r="H5" s="11" t="str">
-        <x:v>ChatGPT</x:v>
-      </x:c>
-      <x:c r="I5" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="J5" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K5" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L5" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="M5" s="11" t="str"/>
+      <x:c r="A5" s="11"/>
+      <x:c r="B5" s="11"/>
+      <x:c r="C5" s="11"/>
+      <x:c r="D5" s="11"/>
+      <x:c r="E5" s="11"/>
+      <x:c r="F5" s="11"/>
+      <x:c r="G5" s="11"/>
+      <x:c r="H5" s="11"/>
+      <x:c r="I5" s="11"/>
+      <x:c r="J5" s="11"/>
+      <x:c r="K5" s="11"/>
+      <x:c r="L5" s="11"/>
+      <x:c r="M5" s="11"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="11" t="str">
-        <x:v>2026-06-29</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="str">
-        <x:v>17:10</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="str">
-        <x:v>DOC-001</x:v>
-      </x:c>
-      <x:c r="D6" s="11" t="str">
-        <x:v>Documentation</x:v>
-      </x:c>
-      <x:c r="E6" s="11" t="str">
-        <x:v>AGENTS.md</x:v>
-      </x:c>
-      <x:c r="F6" s="11" t="str">
-        <x:v>修改</x:v>
-      </x:c>
-      <x:c r="G6" s="11" t="str">
-        <x:v>套用使用者提供的最新 AGENTS.md</x:v>
-      </x:c>
-      <x:c r="H6" s="11" t="str">
-        <x:v>ChatGPT</x:v>
-      </x:c>
-      <x:c r="I6" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="J6" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="K6" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="L6" s="11" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="M6" s="11" t="str"/>
+      <x:c r="A6" s="11"/>
+      <x:c r="B6" s="11"/>
+      <x:c r="C6" s="11"/>
+      <x:c r="D6" s="11"/>
+      <x:c r="E6" s="11"/>
+      <x:c r="F6" s="11"/>
+      <x:c r="G6" s="11"/>
+      <x:c r="H6" s="11"/>
+      <x:c r="I6" s="11"/>
+      <x:c r="J6" s="11"/>
+      <x:c r="K6" s="11"/>
+      <x:c r="L6" s="11"/>
+      <x:c r="M6" s="11"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1078a95c00444163"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refafa90548f64c55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(auth): add refresh session families
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R0464abf6bbab4e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R7b23fa9b13f743f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,6 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
@@ -45,7 +48,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -69,6 +72,25 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -78,7 +100,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M6" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="時間"/>
@@ -94,7 +116,7 @@
     <x:tableColumn id="12" name="是否需要 Migration"/>
     <x:tableColumn id="13" name="備註"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -249,20 +271,20 @@
   <x:cols>
     <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="8" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="54" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="50" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="10" t="str">
         <x:v>日期</x:v>
       </x:c>
@@ -303,85 +325,413 @@
         <x:v>備註</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="11"/>
-      <x:c r="B2" s="11"/>
-      <x:c r="C2" s="11"/>
-      <x:c r="D2" s="11"/>
-      <x:c r="E2" s="11"/>
-      <x:c r="F2" s="11"/>
-      <x:c r="G2" s="11"/>
-      <x:c r="H2" s="11"/>
-      <x:c r="I2" s="11"/>
-      <x:c r="J2" s="11"/>
-      <x:c r="K2" s="11"/>
-      <x:c r="L2" s="11"/>
-      <x:c r="M2" s="11"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="11"/>
-      <x:c r="B3" s="11"/>
-      <x:c r="C3" s="11"/>
-      <x:c r="D3" s="11"/>
-      <x:c r="E3" s="11"/>
-      <x:c r="F3" s="11"/>
-      <x:c r="G3" s="11"/>
-      <x:c r="H3" s="11"/>
-      <x:c r="I3" s="11"/>
-      <x:c r="J3" s="11"/>
-      <x:c r="K3" s="11"/>
-      <x:c r="L3" s="11"/>
-      <x:c r="M3" s="11"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="11"/>
-      <x:c r="B4" s="11"/>
-      <x:c r="C4" s="11"/>
-      <x:c r="D4" s="11"/>
-      <x:c r="E4" s="11"/>
-      <x:c r="F4" s="11"/>
-      <x:c r="G4" s="11"/>
-      <x:c r="H4" s="11"/>
-      <x:c r="I4" s="11"/>
-      <x:c r="J4" s="11"/>
-      <x:c r="K4" s="11"/>
-      <x:c r="L4" s="11"/>
-      <x:c r="M4" s="11"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="11"/>
-      <x:c r="B5" s="11"/>
-      <x:c r="C5" s="11"/>
-      <x:c r="D5" s="11"/>
-      <x:c r="E5" s="11"/>
-      <x:c r="F5" s="11"/>
-      <x:c r="G5" s="11"/>
-      <x:c r="H5" s="11"/>
-      <x:c r="I5" s="11"/>
-      <x:c r="J5" s="11"/>
-      <x:c r="K5" s="11"/>
-      <x:c r="L5" s="11"/>
-      <x:c r="M5" s="11"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="11"/>
-      <x:c r="B6" s="11"/>
-      <x:c r="C6" s="11"/>
-      <x:c r="D6" s="11"/>
-      <x:c r="E6" s="11"/>
-      <x:c r="F6" s="11"/>
-      <x:c r="G6" s="11"/>
-      <x:c r="H6" s="11"/>
-      <x:c r="I6" s="11"/>
-      <x:c r="J6" s="11"/>
-      <x:c r="K6" s="11"/>
-      <x:c r="L6" s="11"/>
-      <x:c r="M6" s="11"/>
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A2" s="16" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B2" s="17" t="str">
+        <x:v>20:31</x:v>
+      </x:c>
+      <x:c r="C2" s="18" t="str">
+        <x:v>REGISTRATION-LOGIN-07</x:v>
+      </x:c>
+      <x:c r="D2" s="18" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E2" s="18" t="str">
+        <x:v>backend/src/main/java/com/monsters/service/session與security/session</x:v>
+      </x:c>
+      <x:c r="F2" s="18" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G2" s="18" t="str">
+        <x:v>建立每次登入獨立Opaque Refresh Session Family及10秒相同結果輪替</x:v>
+      </x:c>
+      <x:c r="H2" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I2" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J2" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K2" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L2" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M2" s="18" t="str">
+        <x:v>Credential只保存SHA-256且後續值以獨立HMAC Secret推導</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="16" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B3" s="17" t="str">
+        <x:v>20:31</x:v>
+      </x:c>
+      <x:c r="C3" s="18" t="str">
+        <x:v>REGISTRATION-LOGIN-07</x:v>
+      </x:c>
+      <x:c r="D3" s="18" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
+        <x:v>JwtTokenService與JwtAuthenticationFilter</x:v>
+      </x:c>
+      <x:c r="F3" s="18" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G3" s="18" t="str">
+        <x:v>核發10分鐘最小claims Access JWT並以sid即時檢查Session</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I3" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J3" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K3" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L3" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M3" s="18" t="str">
+        <x:v>JWT不含Email且reuse撤銷後舊Access立即失效</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="16" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B4" s="17" t="str">
+        <x:v>20:31</x:v>
+      </x:c>
+      <x:c r="C4" s="18" t="str">
+        <x:v>REGISTRATION-LOGIN-07</x:v>
+      </x:c>
+      <x:c r="D4" s="18" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="E4" s="18" t="str">
+        <x:v>backend/src/main/resources/db/migration/V5__add_refresh_session_families.sql</x:v>
+      </x:c>
+      <x:c r="F4" s="18" t="str">
+        <x:v>新增</x:v>
+      </x:c>
+      <x:c r="G4" s="18" t="str">
+        <x:v>建立user_sessions refresh_session_credentials及session_security_audits</x:v>
+      </x:c>
+      <x:c r="H4" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I4" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J4" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K4" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L4" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M4" s="18" t="str">
+        <x:v>空庫與V2升級至V5測試通過</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="16" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>20:31</x:v>
+      </x:c>
+      <x:c r="C5" s="18" t="str">
+        <x:v>REGISTRATION-LOGIN-07</x:v>
+      </x:c>
+      <x:c r="D5" s="18" t="str">
+        <x:v>API</x:v>
+      </x:c>
+      <x:c r="E5" s="18" t="str">
+        <x:v>SessionRefreshController與registration-login.yaml</x:v>
+      </x:c>
+      <x:c r="F5" s="18" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G5" s="18" t="str">
+        <x:v>新增POST api v1 auth session-refreshes及穩定401錯誤碼</x:v>
+      </x:c>
+      <x:c r="H5" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I5" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J5" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K5" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L5" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M5" s="18" t="str">
+        <x:v>無效過期撤銷為AUTH_SESSION_INVALID且reuse為AUTH_REFRESH_REUSE_DETECTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="16" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>20:31</x:v>
+      </x:c>
+      <x:c r="C6" s="18" t="str">
+        <x:v>REGISTRATION-LOGIN-07</x:v>
+      </x:c>
+      <x:c r="D6" s="18" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="E6" s="18" t="str">
+        <x:v>frontend/lib/repositories/auth_repository.dart</x:v>
+      </x:c>
+      <x:c r="F6" s="18" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G6" s="18" t="str">
+        <x:v>將暫時Credential換發切換至v1 Session Refresh API</x:v>
+      </x:c>
+      <x:c r="H6" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I6" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J6" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K6" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L6" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M6" s="18" t="str">
+        <x:v>安全Credential Store留待Task08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="16" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>20:31</x:v>
+      </x:c>
+      <x:c r="C7" s="18" t="str">
+        <x:v>REGISTRATION-LOGIN-07</x:v>
+      </x:c>
+      <x:c r="D7" s="18" t="str">
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="E7" s="18" t="str">
+        <x:v>backend與frontend測試</x:v>
+      </x:c>
+      <x:c r="F7" s="18" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G7" s="18" t="str">
+        <x:v>TDD驗證rotation grace reuse containment期限Security Filter Migration OpenAPI及Repository</x:v>
+      </x:c>
+      <x:c r="H7" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I7" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J7" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K7" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L7" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M7" s="18" t="str">
+        <x:v>Backend單元316與MySQL31及Flutter185項 Analyze Web Build通過</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="16" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>20:31</x:v>
+      </x:c>
+      <x:c r="C8" s="18" t="str">
+        <x:v>REGISTRATION-LOGIN-07</x:v>
+      </x:c>
+      <x:c r="D8" s="18" t="str">
+        <x:v>Dependency</x:v>
+      </x:c>
+      <x:c r="E8" s="18" t="str">
+        <x:v>backend/build.gradle與SmtpEmailDeliveryAdapter</x:v>
+      </x:c>
+      <x:c r="F8" s="18" t="str">
+        <x:v>驗證</x:v>
+      </x:c>
+      <x:c r="G8" s="18" t="str">
+        <x:v>確認Spring Mail starter及SimpleMailMessage與JavaMailSender imports可乾淨編譯</x:v>
+      </x:c>
+      <x:c r="H8" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I8" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J8" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K8" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L8" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M8" s="18" t="str">
+        <x:v>無需加入重複dependency且應由IDE重新載入backend Gradle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="16" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>20:31</x:v>
+      </x:c>
+      <x:c r="C9" s="18" t="str">
+        <x:v>REGISTRATION-LOGIN-07</x:v>
+      </x:c>
+      <x:c r="D9" s="18" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="E9" s="18" t="str">
+        <x:v>README docs Task與Log</x:v>
+      </x:c>
+      <x:c r="F9" s="18" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G9" s="18" t="str">
+        <x:v>同步Session Family契約環境設定Task07 REVIEW及一個月保存期限</x:v>
+      </x:c>
+      <x:c r="H9" s="18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I9" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J9" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K9" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L9" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M9" s="18" t="str">
+        <x:v>截止2026-07-01無超過一個月紀錄</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10"/>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
+      <x:c r="G10"/>
+      <x:c r="H10"/>
+      <x:c r="I10"/>
+      <x:c r="J10"/>
+      <x:c r="K10"/>
+      <x:c r="L10"/>
+      <x:c r="M10"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11"/>
+      <x:c r="B11"/>
+      <x:c r="C11"/>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11"/>
+      <x:c r="I11"/>
+      <x:c r="J11"/>
+      <x:c r="K11"/>
+      <x:c r="L11"/>
+      <x:c r="M11"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12"/>
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
+      <x:c r="I12"/>
+      <x:c r="J12"/>
+      <x:c r="K12"/>
+      <x:c r="L12"/>
+      <x:c r="M12"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
+      <x:c r="K13"/>
+      <x:c r="L13"/>
+      <x:c r="M13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
+      <x:c r="K14"/>
+      <x:c r="L14"/>
+      <x:c r="M14"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refafa90548f64c55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45dc84ada8df46a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record task 07 ci results
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R7b23fa9b13f743f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R2ffee58b7d744803"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -568,7 +568,7 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="M7" s="18" t="str">
-        <x:v>Backend單元316與MySQL31及Flutter185項 Analyze Web Build通過</x:v>
+        <x:v>Backend單元316與MySQL31及Flutter185項 Analyze Web Build通過且PR96四項CI全綠</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -650,7 +650,7 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="M9" s="18" t="str">
-        <x:v>截止2026-07-01無超過一個月紀錄</x:v>
+        <x:v>Draft PR #96四項CI全綠且截止2026-07-01無過期紀錄</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -731,7 +731,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45dc84ada8df46a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc290df113ddb45be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(auth): add platform credential stores
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R2ffee58b7d744803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R653d69f84ee343ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="時間"/>
@@ -654,84 +654,296 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10"/>
-      <x:c r="B10"/>
-      <x:c r="C10"/>
-      <x:c r="D10"/>
-      <x:c r="E10"/>
-      <x:c r="F10"/>
-      <x:c r="G10"/>
-      <x:c r="H10"/>
-      <x:c r="I10"/>
-      <x:c r="J10"/>
-      <x:c r="K10"/>
-      <x:c r="L10"/>
-      <x:c r="M10"/>
+      <x:c r="A10" s="13" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>16:57</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>REGISTRATION-LOGIN-08</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>WebSessionCookieService與Auth Controllers</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>建立Web Cookie transport並驗證可信Origin與CSRF proof</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>Web response不暴露Refresh且無效401清除Cookie</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11"/>
-      <x:c r="B11"/>
-      <x:c r="C11"/>
-      <x:c r="D11"/>
-      <x:c r="E11"/>
-      <x:c r="F11"/>
-      <x:c r="G11"/>
-      <x:c r="H11"/>
-      <x:c r="I11"/>
-      <x:c r="J11"/>
-      <x:c r="K11"/>
-      <x:c r="L11"/>
-      <x:c r="M11"/>
+      <x:c r="A11" s="13" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>16:57</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>REGISTRATION-LOGIN-08</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>auth_session_store與auth_repository及Splash</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>建立Web Android iOS Credential Store及安全恢復失敗流程</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>Access只存記憶體且SharedPreferences不存LoginResult</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12"/>
-      <x:c r="B12"/>
-      <x:c r="C12"/>
-      <x:c r="D12"/>
-      <x:c r="E12"/>
-      <x:c r="F12"/>
-      <x:c r="G12"/>
-      <x:c r="H12"/>
-      <x:c r="I12"/>
-      <x:c r="J12"/>
-      <x:c r="K12"/>
-      <x:c r="L12"/>
-      <x:c r="M12"/>
+      <x:c r="A12" s="13" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>16:57</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>REGISTRATION-LOGIN-08</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Dependency</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>frontend pubspec與Android設定</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>加入flutter_secure_storage 10.3.1並設定Android API23與停用備份</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>iOS Keychain不同步且不可跨裝置遷移</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13"/>
-      <x:c r="B13"/>
-      <x:c r="C13"/>
-      <x:c r="D13"/>
-      <x:c r="E13"/>
-      <x:c r="F13"/>
-      <x:c r="G13"/>
-      <x:c r="H13"/>
-      <x:c r="I13"/>
-      <x:c r="J13"/>
-      <x:c r="K13"/>
-      <x:c r="L13"/>
-      <x:c r="M13"/>
+      <x:c r="A13" s="13" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>16:57</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>REGISTRATION-LOGIN-08</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>backend與frontend測試</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>TDD驗證Cookie CSRF三平台Store single flight與暫時錯誤</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>Backend316與MySQL36 Flutter190項及Analyze通過</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14"/>
-      <x:c r="B14"/>
-      <x:c r="C14"/>
-      <x:c r="D14"/>
-      <x:c r="E14"/>
-      <x:c r="F14"/>
-      <x:c r="G14"/>
-      <x:c r="H14"/>
-      <x:c r="I14"/>
-      <x:c r="J14"/>
-      <x:c r="K14"/>
-      <x:c r="L14"/>
-      <x:c r="M14"/>
+      <x:c r="A14" s="13" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>16:57</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>REGISTRATION-LOGIN-08</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Build</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Flutter Web與Android</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>驗證</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>完成Web release與Android debug APK build</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>Android損壞增量cache清理後以非增量fallback成功</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>16:57</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>REGISTRATION-LOGIN-08</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>README規格OpenAPI與Task</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>同步三平台Session契約設定決策並將Task08轉REVIEW</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>Database無異動且Task07依PR96證據轉DONE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>16:57</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>REGISTRATION-LOGIN-08</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>log CHANGE_LOG與CHANGE_HISTORY</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>新增Task08工作報告並清除一個月前Log</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>移除Jul1至Jul2共13區段與99筆CSV紀錄並正規化41筆舊9欄紀錄</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc290df113ddb45be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad36195e38724bd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(auth): record Task 08 CI evidence
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R653d69f84ee343ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R66dc80d2c54f4ba3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="時間"/>
@@ -940,10 +940,92 @@
         <x:v>移除Jul1至Jul2共13區段與99筆CSV紀錄並正規化41筆舊9欄紀錄</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="n">
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>09:40</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>REGISTRATION-LOGIN-08-REVIEW</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>.github/workflows/registration-login-ci.yml與frontend/android/app/build.gradle.kts</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>修改與驗證</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>加入Flutter 3.29.2 Android APK Build並依Plugin需求調整Android平台門檻</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>PR #97四項CI全綠；最低API24 compileSdk36 NDK27且本機APK通過</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="13" t="n">
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>09:40</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>REGISTRATION-LOGIN-08-REVIEW</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>docs規格Task與log三種歷史紀錄</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>同步方案A平台決策PR與CI證據並執行一個月Log保存期限清理</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>移除7月10日前22個Markdown區段與278筆CSV；Task08維持REVIEW</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad36195e38724bd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0ea0960f6dc4e92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): add static responsive showcase
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R66dc80d2c54f4ba3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="Rfa1cb14cd6a64dbe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="時間"/>
@@ -1022,10 +1022,92 @@
         <x:v>移除7月10日前22個Markdown區段與278筆CSV；Task08維持REVIEW</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="13" t="n">
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>10:16</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>UI-SHOWCASE-HTML</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>docs/ui-showcase/index.html</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>新增與驗證</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>建立純HTML已完成畫面展示並內嵌Mobile Tablet Desktop RWD與頁面錨點連結</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K19" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L19" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>無API JavaScript邏輯判斷動畫或真實會員資料；120個連結均有效</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="13" t="n">
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>10:16</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>UI-SHOWCASE-HTML</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>docs/UI_SPEC.md、docs/TASKS.md與log三種歷史紀錄</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>同步靜態展示範圍RWD限制驗證證據與一個月Log保存期限檢查</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K20" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L20" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M20" t="str">
+        <x:v>截止2026-07-10無過期紀錄；未修改system_data</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0ea0960f6dc4e92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R712137eefb314070"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(auth): 支援跨站 Web Session Cookie
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="Rfa1cb14cd6a64dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R3bd8fa3efbd4454d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="時間"/>
@@ -1104,10 +1104,174 @@
         <x:v>截止2026-07-10無過期紀錄；未修改system_data</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="13" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>07:43</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>REG-LOGIN-08-CROSS-SITE</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>WebSessionCookieService與AuthMemberHttpIntegrationTest</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>將Web Refresh Cookie改為SameSite None Secure支援Pages至Railway跨站HTTPS</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L21" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>仍強制可信Origin CORS與CSRF custom header</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="13" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>07:43</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>REG-LOGIN-08-CROSS-SITE</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>frontend/test/core/network/api_client_test.dart</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>明確驗證每個401原Request換發後最多重試一次</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K22" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L22" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>Backend316 MySQL36 Flutter191項及Analyze通過</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="13" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>07:43</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>REG-LOGIN-08-CROSS-SITE</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Git</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>feature/phase4.5-secure-session-store</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>同步</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>快轉至已含PR97與PR98的最新feature phase4.5並保留遠端成果</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K23" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L23" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>未以舊基底覆蓋整合測試Android設定或UI展示頁</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="13" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>07:43</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>REG-LOGIN-08-CROSS-SITE</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>README docs Task與Log</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>修改</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>同步跨站Cookie決策Task08 DONE及一個月Log保存期限</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K24" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>刪除39個Markdown區段與479筆CSV且XLSX無過期資料</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R712137eefb314070"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2dca294f20240c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(auth): 記錄跨站 Session CI 結果
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R3bd8fa3efbd4454d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R1e04e14d97814888"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1183,7 +1183,7 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="M22" t="str">
-        <x:v>Backend316 MySQL36 Flutter191項及Analyze通過</x:v>
+        <x:v>PR99 Backend MySQL Flutter加Android及OpenAPI四項CI全綠</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1271,7 +1271,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2dca294f20240c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra99e6283c817454e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(auth): 記錄 Task 09 Draft PR
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R16a6d64dbcc74c05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R180dc6d74d2d433d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1552,13 +1552,13 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="M31" t="str">
-        <x:v>截止2026-07-16無過期Log；system_data保持唯讀</x:v>
+        <x:v>Draft PR100已建立；截止2026-07-16無過期Log且system_data唯讀</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6e8918b2c8240ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fe76c6dc9784959"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(auth): 記錄 Task 10 PR 驗證結果
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="Rcf0d3c7169cb46bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R37092e70b7b44afc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1798,7 +1798,7 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="M37" t="str">
-        <x:v>Backend 321項與MySQL 39項；Flutter 209項 Analyze Web及Android build通過</x:v>
+        <x:v>Backend 321與MySQL 39；Flutter 209 Analyze Web Android及PR101四項CI通過</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -1839,13 +1839,13 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="M38" t="str">
-        <x:v>刪除2026-07-16至07-19過期Markdown與CSV Log；XLSX無過期列</x:v>
+        <x:v>Draft PR101四項CI全綠；已清除過期Markdown與CSV且XLSX無過期列</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c01ec508f04653"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7782c449fac0477f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(auth): record password reset review evidence
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R37092e70b7b44afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R9e38c1f574f4400a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="時間"/>
@@ -284,7 +284,7 @@
     <x:col min="13" max="13" width="50" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
+    <x:row r="1" ht="30" hidden="0" customHeight="1">
       <x:c r="A1" s="10" t="str">
         <x:v>日期</x:v>
       </x:c>
@@ -1842,10 +1842,420 @@
         <x:v>Draft PR101四項CI全綠；已清除過期Markdown與CSV且XLSX無過期列</x:v>
       </x:c>
     </x:row>
+    <x:row r="39" ht="36" customHeight="1">
+      <x:c r="A39" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B39" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C39" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D39" s="11" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E39" s="11" t="str">
+        <x:v>PasswordReset controller/service/worker與session</x:v>
+      </x:c>
+      <x:c r="F39" s="11" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G39" s="11" t="str">
+        <x:v>通用202受理與可靠寄信；15分鐘單次Token只存hash；成功撤銷全部Session</x:v>
+      </x:c>
+      <x:c r="H39" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I39" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J39" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K39" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L39" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M39" s="11" t="str">
+        <x:v>採方案1；不回傳reset Token；失敗重試與無PII告警</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="36" customHeight="1">
+      <x:c r="A40" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B40" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C40" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D40" s="11" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="E40" s="11" t="str">
+        <x:v>V9__formalize_password_reset.sql</x:v>
+      </x:c>
+      <x:c r="F40" s="11" t="str">
+        <x:v>新增</x:v>
+      </x:c>
+      <x:c r="G40" s="11" t="str">
+        <x:v>token_hash上限64；新增revoked_at與active查詢索引</x:v>
+      </x:c>
+      <x:c r="H40" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I40" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J40" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K40" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L40" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M40" s="11" t="str">
+        <x:v>沿用既有表；舊Migration不改寫；Registration升級斷言由V8校正為V9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="36" customHeight="1">
+      <x:c r="A41" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B41" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C41" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D41" s="11" t="str">
+        <x:v>API</x:v>
+      </x:c>
+      <x:c r="E41" s="11" t="str">
+        <x:v>API_SPEC與registration-login.yaml</x:v>
+      </x:c>
+      <x:c r="F41" s="11" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G41" s="11" t="str">
+        <x:v>新增password-reset-requests與password-resets兩組v1契約</x:v>
+      </x:c>
+      <x:c r="H41" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I41" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J41" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K41" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L41" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M41" s="11" t="str">
+        <x:v>舊路徑暫留安全deprecated別名，Task18驗收後移除</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="36" customHeight="1">
+      <x:c r="A42" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B42" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C42" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D42" s="11" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="E42" s="11" t="str">
+        <x:v>PasswordReset頁面/provider/repository/router</x:v>
+      </x:c>
+      <x:c r="F42" s="11" t="str">
+        <x:v>新增與修改</x:v>
+      </x:c>
+      <x:c r="G42" s="11" t="str">
+        <x:v>完成申請、受理、Token失效與成功頁；修正鍵盤避讓及舊回應隔離</x:v>
+      </x:c>
+      <x:c r="H42" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I42" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J42" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K42" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L42" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M42" s="11" t="str">
+        <x:v>390至1920 RWD；矮視窗收合；NFC長度交Backend判定；換Token清空舊狀態</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="36" customHeight="1">
+      <x:c r="A43" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B43" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C43" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D43" s="11" t="str">
+        <x:v>Penpot</x:v>
+      </x:c>
+      <x:c r="E43" s="11" t="str">
+        <x:v>WEB與APP主畫板及Password Reset狀態</x:v>
+      </x:c>
+      <x:c r="F43" s="11" t="str">
+        <x:v>新增與整理</x:v>
+      </x:c>
+      <x:c r="G43" s="11" t="str">
+        <x:v>新增Web/Mobile共16狀態；35主畫板分區且無重疊；466元件位置尺寸不變</x:v>
+      </x:c>
+      <x:c r="H43" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I43" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J43" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K43" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L43" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M43" s="11" t="str">
+        <x:v>180個descendant containment通過；Chrome截圖已檢視；未刪舊畫板及素材</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="36" customHeight="1">
+      <x:c r="A44" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B44" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C44" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D44" s="11" t="str">
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="E44" s="11" t="str">
+        <x:v>Backend與Flutter測試及建置</x:v>
+      </x:c>
+      <x:c r="F44" s="11" t="str">
+        <x:v>驗證</x:v>
+      </x:c>
+      <x:c r="G44" s="11" t="str">
+        <x:v>Backend單元324通過4跳過；MySQL42通過；Flutter236通過且Analyze無問題</x:v>
+      </x:c>
+      <x:c r="H44" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I44" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J44" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K44" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L44" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M44" s="11" t="str">
+        <x:v>Web release與Android debug成功；本機Flutter3.44.6；CI3.29.2待PR觸發</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="36" customHeight="1">
+      <x:c r="A45" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B45" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C45" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D45" s="11" t="str">
+        <x:v>Cleanup</x:v>
+      </x:c>
+      <x:c r="E45" s="11" t="str">
+        <x:v>PASSWORD_RESET_LEGACY_CLEANUP與舊DTO</x:v>
+      </x:c>
+      <x:c r="F45" s="11" t="str">
+        <x:v>刪除與文件化</x:v>
+      </x:c>
+      <x:c r="G45" s="11" t="str">
+        <x:v>移除raw Token response、舊AuthService方法及3個DTO；列出後續刪除條件</x:v>
+      </x:c>
+      <x:c r="H45" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I45" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J45" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K45" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L45" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M45" s="11" t="str">
+        <x:v>system_data與其他legacy登入流程未刪除；可由Git取回本次移除檔案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="36" customHeight="1">
+      <x:c r="A46" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B46" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C46" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D46" s="11" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="E46" s="11" t="str">
+        <x:v>Task與Project/API/Database/UI/README/DECISIONS</x:v>
+      </x:c>
+      <x:c r="F46" s="11" t="str">
+        <x:v>同步</x:v>
+      </x:c>
+      <x:c r="G46" s="11" t="str">
+        <x:v>Task10依PR101合併證據標DONE；Task11由IN PROGRESS轉REVIEW</x:v>
+      </x:c>
+      <x:c r="H46" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I46" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J46" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K46" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L46" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M46" s="11" t="str">
+        <x:v>待提交Draft PR/CI/使用者Review與合併；不宣告DONE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="36" customHeight="1">
+      <x:c r="A47" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B47" s="11" t="str">
+        <x:v>14:40</x:v>
+      </x:c>
+      <x:c r="C47" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D47" s="11" t="str">
+        <x:v>Log</x:v>
+      </x:c>
+      <x:c r="E47" s="11" t="str">
+        <x:v>CHANGE_LOG與CHANGE_HISTORY</x:v>
+      </x:c>
+      <x:c r="F47" s="11" t="str">
+        <x:v>保存期限清理</x:v>
+      </x:c>
+      <x:c r="G47" s="11" t="str">
+        <x:v>保留2026-07-31起紀錄；移除20段Markdown及124筆CSV過期紀錄</x:v>
+      </x:c>
+      <x:c r="H47" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I47" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J47" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K47" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L47" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M47" s="11" t="str">
+        <x:v>XLSX無過期列；保留既有表格樣式；已刪Log可由Git歷史取回</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="48" customHeight="1">
+      <x:c r="A48" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B48" s="11" t="str">
+        <x:v>14:48</x:v>
+      </x:c>
+      <x:c r="C48" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D48" s="11" t="str">
+        <x:v>Git</x:v>
+      </x:c>
+      <x:c r="E48" s="11" t="str">
+        <x:v>Task11功能與三份Log</x:v>
+      </x:c>
+      <x:c r="F48" s="11" t="str">
+        <x:v>提交紀錄</x:v>
+      </x:c>
+      <x:c r="G48" s="11" t="str">
+        <x:v>功能提交0829f5d；Log同步提交後一併推送Task分支</x:v>
+      </x:c>
+      <x:c r="H48" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I48" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J48" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K48" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L48" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M48" s="11" t="str">
+        <x:v>feature/phase4.5-password-reset → feature/phase4.5；Draft PR送審，不自動合併</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7782c449fac0477f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75666e3a4393455d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ui): align password reset logos with Penpot
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R9e38c1f574f4400a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="Re5a1ed65b39e4873"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeHistoryTable" displayName="ChangeHistoryTable" ref="A1:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="時間"/>
@@ -2252,10 +2252,51 @@
         <x:v>feature/phase4.5-password-reset → feature/phase4.5；Draft PR送審，不自動合併</x:v>
       </x:c>
     </x:row>
+    <x:row r="49" ht="48" customHeight="1">
+      <x:c r="A49" s="12" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B49" s="11" t="str">
+        <x:v>15:00</x:v>
+      </x:c>
+      <x:c r="C49" s="11" t="str">
+        <x:v>REGISTRATION-LOGIN-11</x:v>
+      </x:c>
+      <x:c r="D49" s="11" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="E49" s="11" t="str">
+        <x:v>PasswordReset三個共用元件/測試/UI規格</x:v>
+      </x:c>
+      <x:c r="F49" s="11" t="str">
+        <x:v>視覺校正</x:v>
+      </x:c>
+      <x:c r="G49" s="11" t="str">
+        <x:v>Logo依Penpot固定150×47與160×50，補Mobile/Desktop尺寸斷言</x:v>
+      </x:c>
+      <x:c r="H49" s="11" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I49" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J49" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="K49" s="11" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L49" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="M49" s="11" t="str">
+        <x:v>PR102；27項專項測試通過；Web重建通過；最新CI於Push後重跑，仍為REVIEW</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75666e3a4393455d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra981aed7d7a84ab6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(member): record Task 12 review evidence
</commit_message>
<xml_diff>
--- a/log/CHANGE_HISTORY.xlsx
+++ b/log/CHANGE_HISTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="Rd7416f5217734297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="1" r:id="R8b1fc29351fc480d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2290,13 +2290,13 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="M49" s="11" t="str">
-        <x:v>移除2026-08-03前Markdown6段 CSV39筆 XLSX8筆；PR與CI完成前不轉DONE</x:v>
+        <x:v>功能提交528c262；Task12 REVIEW；推送feature/phase4.5-member-data-modification並建立至feature/phase4.5的Draft PR；不自動合併</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3a12a348ac740c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0acacbd66e764ca9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>